<commit_message>
Refine OG0060 hint and distractor
</commit_message>
<xml_diff>
--- a/v3/OG0060/OG0060_DevSpec.xlsx
+++ b/v3/OG0060/OG0060_DevSpec.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METADATA" sheetId="1" r:id="R8513d725dc304f26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUESTION_SPEC" sheetId="2" r:id="Re03186d2d468482b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASSETS" sheetId="3" r:id="Rf29b5e3f82204cee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESPONSE_QUALITY" sheetId="4" r:id="R88d8aafe342c4ad5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METADATA" sheetId="1" r:id="R9619195914964b67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUESTION_SPEC" sheetId="2" r:id="Rfd08debe5e814a63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASSETS" sheetId="3" r:id="Rbc3df50903ed4c07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESPONSE_QUALITY" sheetId="4" r:id="Rf96fb3070f4f4020"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>